<commit_message>
Sort deals most-recent-first within sector; rebuild 31-Jul-26 workbook
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01LRozwLgExAwjo3Y71TMLZS
</commit_message>
<xml_diff>
--- a/weekly-deals/outputs/Weekly_Fintech_Deals_2026-07-31.xlsx
+++ b/weekly-deals/outputs/Weekly_Fintech_Deals_2026-07-31.xlsx
@@ -687,37 +687,31 @@
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>27-Jul-26</t>
+          <t>30-Jul-26</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>Water Street Labs &amp; CX Clearinghouse</t>
+          <t>MarketAxess</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
         <is>
-          <t>Fanatics</t>
-        </is>
-      </c>
-      <c r="I3" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="J3" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="K3" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+          <t>Intercontinental Exchange</t>
+        </is>
+      </c>
+      <c r="I3" s="2" t="n">
+        <v>5700</v>
+      </c>
+      <c r="J3" s="4" t="n">
+        <v>6.5</v>
+      </c>
+      <c r="K3" s="4" t="n">
+        <v>13</v>
       </c>
       <c r="L3" s="2" t="inlineStr">
         <is>
-          <t>CFTC-registered designated contract market and derivatives clearinghouse letting Fanatics Markets self-list and self-clear sports and event prediction contracts</t>
+          <t>Electronic fixed-income trading marketplace (all-to-all Open Trading liquidity, RFQ protocols) with bond pricing data and execution-automation tools; all-cash take-private at $167.00/share, a 33% premium</t>
         </is>
       </c>
       <c r="M3" s="3" t="inlineStr">
@@ -727,17 +721,17 @@
       </c>
       <c r="N3" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>ICE press release; MKTX 4Q25/2Q26 earnings; deal press (EBITDA)</t>
         </is>
       </c>
       <c r="O3" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>EV ~$5.7B (equity ~$6.0B); LTM Jun-26 rev ~$872M (FY25 $846M + H1'26 $452M - H1'25 ~$426M); LTM adj. EBITDA ~$438M implied from reported ~10.6x synergized multiple less $100M run-rate synergies</t>
         </is>
       </c>
       <c r="P3" s="2" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="Q3" s="2" t="inlineStr">
@@ -747,7 +741,7 @@
       </c>
       <c r="R3" s="2" t="inlineStr">
         <is>
-          <t>BGC Group</t>
+          <t>-</t>
         </is>
       </c>
     </row>
@@ -775,31 +769,37 @@
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>30-Jul-26</t>
+          <t>27-Jul-26</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>MarketAxess</t>
+          <t>Water Street Labs &amp; CX Clearinghouse</t>
         </is>
       </c>
       <c r="H4" s="2" t="inlineStr">
         <is>
-          <t>Intercontinental Exchange</t>
-        </is>
-      </c>
-      <c r="I4" s="2" t="n">
-        <v>5700</v>
-      </c>
-      <c r="J4" s="4" t="n">
-        <v>6.5</v>
-      </c>
-      <c r="K4" s="4" t="n">
-        <v>13</v>
+          <t>Fanatics</t>
+        </is>
+      </c>
+      <c r="I4" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J4" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K4" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
       <c r="L4" s="2" t="inlineStr">
         <is>
-          <t>Electronic fixed-income trading marketplace (all-to-all Open Trading liquidity, RFQ protocols) with bond pricing data and execution-automation tools; all-cash take-private at $167.00/share, a 33% premium</t>
+          <t>CFTC-registered designated contract market and derivatives clearinghouse letting Fanatics Markets self-list and self-clear sports and event prediction contracts</t>
         </is>
       </c>
       <c r="M4" s="3" t="inlineStr">
@@ -809,17 +809,17 @@
       </c>
       <c r="N4" s="2" t="inlineStr">
         <is>
-          <t>ICE press release; MKTX 4Q25/2Q26 earnings; deal press (EBITDA)</t>
+          <t>-</t>
         </is>
       </c>
       <c r="O4" s="2" t="inlineStr">
         <is>
-          <t>EV ~$5.7B (equity ~$6.0B); LTM Jun-26 rev ~$872M (FY25 $846M + H1'26 $452M - H1'25 ~$426M); LTM adj. EBITDA ~$438M implied from reported ~10.6x synergized multiple less $100M run-rate synergies</t>
+          <t>-</t>
         </is>
       </c>
       <c r="P4" s="2" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>N</t>
         </is>
       </c>
       <c r="Q4" s="2" t="inlineStr">
@@ -829,7 +829,7 @@
       </c>
       <c r="R4" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>BGC Group</t>
         </is>
       </c>
     </row>
@@ -1432,21 +1432,21 @@
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>28-Jul-26</t>
+          <t>29-Jul-26</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>PEX</t>
+          <t>Freehand</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>Bluff Point Associates</t>
+          <t>Battery Ventures, NewRoad Capital Partners</t>
         </is>
       </c>
       <c r="H4" s="2" t="n">
-        <v>160</v>
+        <v>75</v>
       </c>
       <c r="I4" s="2" t="inlineStr">
         <is>
@@ -1465,7 +1465,7 @@
       </c>
       <c r="L4" s="2" t="inlineStr">
         <is>
-          <t>Corporate card issuing and spend-management platform for SMBs automating expense controls, reconciliation, and AP; $160M combined equity and debt, with the card facility provided by Clear Haven</t>
+          <t>Autonomous AI agents automating enterprise procure-to-pay — procurement, supplier management, invoice and freight audit, and payments — for Fortune 500 companies</t>
         </is>
       </c>
       <c r="M4" s="3" t="inlineStr">
@@ -1493,21 +1493,21 @@
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>29-Jul-26</t>
+          <t>28-Jul-26</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>Freehand</t>
+          <t>PEX</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>Battery Ventures, NewRoad Capital Partners</t>
+          <t>Bluff Point Associates</t>
         </is>
       </c>
       <c r="H5" s="2" t="n">
-        <v>75</v>
+        <v>160</v>
       </c>
       <c r="I5" s="2" t="inlineStr">
         <is>
@@ -1526,7 +1526,7 @@
       </c>
       <c r="L5" s="2" t="inlineStr">
         <is>
-          <t>Autonomous AI agents automating enterprise procure-to-pay — procurement, supplier management, invoice and freight audit, and payments — for Fortune 500 companies</t>
+          <t>Corporate card issuing and spend-management platform for SMBs automating expense controls, reconciliation, and AP; $160M combined equity and debt, with the card facility provided by Clear Haven</t>
         </is>
       </c>
       <c r="M5" s="3" t="inlineStr">

</xml_diff>